<commit_message>
New plots, new data, and quarterly target added. Also, some code refactoring and cleanup.
</commit_message>
<xml_diff>
--- a/data/output_4.15.26.xlsx
+++ b/data/output_4.15.26.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -417,71 +429,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M81"/>
+  <dimension ref="A1:M89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Board</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Project Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Job #</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Equipment</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>QTY</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Amps</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>LFG ENG</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Design Start Date</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Design End Date</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t># Design Days</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Difficulty</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
@@ -520,10 +532,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I2" s="1" t="n">
+      <c r="I2" s="2" t="n">
         <v>45876</v>
       </c>
-      <c r="J2" s="1" t="n">
+      <c r="J2" s="2" t="n">
         <v>45888</v>
       </c>
       <c r="K2" t="n">
@@ -573,10 +585,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I3" s="1" t="n">
+      <c r="I3" s="2" t="n">
         <v>45887</v>
       </c>
-      <c r="J3" s="1" t="n">
+      <c r="J3" s="2" t="n">
         <v>45901</v>
       </c>
       <c r="K3" t="n">
@@ -626,10 +638,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I4" s="1" t="n">
+      <c r="I4" s="2" t="n">
         <v>45889</v>
       </c>
-      <c r="J4" s="1" t="n">
+      <c r="J4" s="2" t="n">
         <v>45901</v>
       </c>
       <c r="K4" t="n">
@@ -679,10 +691,10 @@
           <t>Shannon</t>
         </is>
       </c>
-      <c r="I5" s="1" t="n">
+      <c r="I5" s="2" t="n">
         <v>45890</v>
       </c>
-      <c r="J5" s="1" t="n">
+      <c r="J5" s="2" t="n">
         <v>45910</v>
       </c>
       <c r="K5" t="n">
@@ -732,10 +744,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I6" s="1" t="n">
+      <c r="I6" s="2" t="n">
         <v>45896</v>
       </c>
-      <c r="J6" s="1" t="n">
+      <c r="J6" s="2" t="n">
         <v>45901</v>
       </c>
       <c r="K6" t="n">
@@ -789,10 +801,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I7" s="1" t="n">
+      <c r="I7" s="2" t="n">
         <v>45897</v>
       </c>
-      <c r="J7" s="1" t="n">
+      <c r="J7" s="2" t="n">
         <v>45908</v>
       </c>
       <c r="K7" t="n">
@@ -842,10 +854,10 @@
           <t>Jacob</t>
         </is>
       </c>
-      <c r="I8" s="1" t="n">
+      <c r="I8" s="2" t="n">
         <v>45905</v>
       </c>
-      <c r="J8" s="1" t="n">
+      <c r="J8" s="2" t="n">
         <v>45912</v>
       </c>
       <c r="K8" t="n">
@@ -899,10 +911,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I9" s="1" t="n">
+      <c r="I9" s="2" t="n">
         <v>45908</v>
       </c>
-      <c r="J9" s="1" t="n">
+      <c r="J9" s="2" t="n">
         <v>45909</v>
       </c>
       <c r="K9" t="n">
@@ -952,10 +964,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I10" s="1" t="n">
+      <c r="I10" s="2" t="n">
         <v>45912</v>
       </c>
-      <c r="J10" s="1" t="n">
+      <c r="J10" s="2" t="n">
         <v>45919</v>
       </c>
       <c r="K10" t="n">
@@ -1005,10 +1017,10 @@
           <t>Jacob</t>
         </is>
       </c>
-      <c r="I11" s="1" t="n">
+      <c r="I11" s="2" t="n">
         <v>45912</v>
       </c>
-      <c r="J11" s="1" t="n">
+      <c r="J11" s="2" t="n">
         <v>45937</v>
       </c>
       <c r="K11" t="n">
@@ -1062,10 +1074,10 @@
           <t>Shannon</t>
         </is>
       </c>
-      <c r="I12" s="1" t="n">
+      <c r="I12" s="2" t="n">
         <v>45918</v>
       </c>
-      <c r="J12" s="1" t="n">
+      <c r="J12" s="2" t="n">
         <v>45933</v>
       </c>
       <c r="K12" t="n">
@@ -1119,10 +1131,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I13" s="1" t="n">
+      <c r="I13" s="2" t="n">
         <v>45919</v>
       </c>
-      <c r="J13" s="1" t="n">
+      <c r="J13" s="2" t="n">
         <v>45921</v>
       </c>
       <c r="K13" t="n">
@@ -1176,10 +1188,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I14" s="1" t="n">
+      <c r="I14" s="2" t="n">
         <v>45924</v>
       </c>
-      <c r="J14" s="1" t="n">
+      <c r="J14" s="2" t="n">
         <v>45929</v>
       </c>
       <c r="K14" t="n">
@@ -1233,10 +1245,10 @@
           <t>Emma</t>
         </is>
       </c>
-      <c r="I15" s="1" t="n">
+      <c r="I15" s="2" t="n">
         <v>45926</v>
       </c>
-      <c r="J15" s="1" t="n">
+      <c r="J15" s="2" t="n">
         <v>46009</v>
       </c>
       <c r="K15" t="n">
@@ -1290,10 +1302,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I16" s="1" t="n">
+      <c r="I16" s="2" t="n">
         <v>45929</v>
       </c>
-      <c r="J16" s="1" t="n">
+      <c r="J16" s="2" t="n">
         <v>45931</v>
       </c>
       <c r="K16" t="n">
@@ -1347,10 +1359,10 @@
           <t>Emma</t>
         </is>
       </c>
-      <c r="I17" s="1" t="n">
+      <c r="I17" s="2" t="n">
         <v>45932</v>
       </c>
-      <c r="J17" s="1" t="n">
+      <c r="J17" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="K17" t="n">
@@ -1404,10 +1416,10 @@
           <t>Shannon</t>
         </is>
       </c>
-      <c r="I18" s="1" t="n">
+      <c r="I18" s="2" t="n">
         <v>45936</v>
       </c>
-      <c r="J18" s="1" t="n">
+      <c r="J18" s="2" t="n">
         <v>45946</v>
       </c>
       <c r="K18" t="n">
@@ -1461,10 +1473,10 @@
           <t>Emma</t>
         </is>
       </c>
-      <c r="I19" s="1" t="n">
+      <c r="I19" s="2" t="n">
         <v>45937</v>
       </c>
-      <c r="J19" s="1" t="n">
+      <c r="J19" s="2" t="n">
         <v>45940</v>
       </c>
       <c r="K19" t="n">
@@ -1518,10 +1530,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I20" s="1" t="n">
+      <c r="I20" s="2" t="n">
         <v>45938</v>
       </c>
-      <c r="J20" s="1" t="n">
+      <c r="J20" s="2" t="n">
         <v>45944</v>
       </c>
       <c r="K20" t="n">
@@ -1571,10 +1583,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I21" s="1" t="n">
+      <c r="I21" s="2" t="n">
         <v>45944</v>
       </c>
-      <c r="J21" s="1" t="n">
+      <c r="J21" s="2" t="n">
         <v>45952</v>
       </c>
       <c r="K21" t="n">
@@ -1628,10 +1640,10 @@
           <t>Shannon</t>
         </is>
       </c>
-      <c r="I22" s="1" t="n">
+      <c r="I22" s="2" t="n">
         <v>45947</v>
       </c>
-      <c r="J22" s="1" t="n">
+      <c r="J22" s="2" t="n">
         <v>45966</v>
       </c>
       <c r="K22" t="n">
@@ -1681,10 +1693,10 @@
           <t>Emma</t>
         </is>
       </c>
-      <c r="I23" s="1" t="n">
+      <c r="I23" s="2" t="n">
         <v>45952</v>
       </c>
-      <c r="J23" s="1" t="n">
+      <c r="J23" s="2" t="n">
         <v>45954</v>
       </c>
       <c r="K23" t="n">
@@ -1734,10 +1746,10 @@
           <t>Emma</t>
         </is>
       </c>
-      <c r="I24" s="1" t="n">
+      <c r="I24" s="2" t="n">
         <v>45952</v>
       </c>
-      <c r="J24" s="1" t="n">
+      <c r="J24" s="2" t="n">
         <v>45954</v>
       </c>
       <c r="K24" t="n">
@@ -1791,10 +1803,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I25" s="1" t="n">
+      <c r="I25" s="2" t="n">
         <v>45952</v>
       </c>
-      <c r="J25" s="1" t="n">
+      <c r="J25" s="2" t="n">
         <v>45958</v>
       </c>
       <c r="K25" t="n">
@@ -1844,10 +1856,10 @@
           <t>Emma</t>
         </is>
       </c>
-      <c r="I26" s="1" t="n">
+      <c r="I26" s="2" t="n">
         <v>45954</v>
       </c>
-      <c r="J26" s="1" t="n">
+      <c r="J26" s="2" t="n">
         <v>45966</v>
       </c>
       <c r="K26" t="n">
@@ -1901,10 +1913,10 @@
           <t>Jacob</t>
         </is>
       </c>
-      <c r="I27" s="1" t="n">
+      <c r="I27" s="2" t="n">
         <v>45957</v>
       </c>
-      <c r="J27" s="1" t="n">
+      <c r="J27" s="2" t="n">
         <v>45967</v>
       </c>
       <c r="K27" t="n">
@@ -1958,10 +1970,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I28" s="1" t="n">
+      <c r="I28" s="2" t="n">
         <v>45958</v>
       </c>
-      <c r="J28" s="1" t="n">
+      <c r="J28" s="2" t="n">
         <v>45966</v>
       </c>
       <c r="K28" t="n">
@@ -2015,10 +2027,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I29" s="1" t="n">
+      <c r="I29" s="2" t="n">
         <v>45958</v>
       </c>
-      <c r="J29" s="1" t="n">
+      <c r="J29" s="2" t="n">
         <v>45966</v>
       </c>
       <c r="K29" t="n">
@@ -2072,10 +2084,10 @@
           <t>Emma</t>
         </is>
       </c>
-      <c r="I30" s="1" t="n">
+      <c r="I30" s="2" t="n">
         <v>45966</v>
       </c>
-      <c r="J30" s="1" t="n">
+      <c r="J30" s="2" t="n">
         <v>45972</v>
       </c>
       <c r="K30" t="n">
@@ -2129,10 +2141,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I31" s="1" t="n">
+      <c r="I31" s="2" t="n">
         <v>45966</v>
       </c>
-      <c r="J31" s="1" t="n">
+      <c r="J31" s="2" t="n">
         <v>45973</v>
       </c>
       <c r="K31" t="n">
@@ -2186,10 +2198,10 @@
           <t>Shannon</t>
         </is>
       </c>
-      <c r="I32" s="1" t="n">
+      <c r="I32" s="2" t="n">
         <v>45966</v>
       </c>
-      <c r="J32" s="1" t="n">
+      <c r="J32" s="2" t="n">
         <v>45980</v>
       </c>
       <c r="K32" t="n">
@@ -2243,10 +2255,10 @@
           <t>Emma</t>
         </is>
       </c>
-      <c r="I33" s="1" t="n">
+      <c r="I33" s="2" t="n">
         <v>45972</v>
       </c>
-      <c r="J33" s="1" t="n">
+      <c r="J33" s="2" t="n">
         <v>45973</v>
       </c>
       <c r="K33" t="n">
@@ -2300,10 +2312,10 @@
           <t>Emma</t>
         </is>
       </c>
-      <c r="I34" s="1" t="n">
+      <c r="I34" s="2" t="n">
         <v>45973</v>
       </c>
-      <c r="J34" s="1" t="n">
+      <c r="J34" s="2" t="n">
         <v>45975</v>
       </c>
       <c r="K34" t="n">
@@ -2357,10 +2369,10 @@
           <t>Shannon</t>
         </is>
       </c>
-      <c r="I35" s="1" t="n">
+      <c r="I35" s="2" t="n">
         <v>45974</v>
       </c>
-      <c r="J35" s="1" t="n">
+      <c r="J35" s="2" t="n">
         <v>45993</v>
       </c>
       <c r="K35" t="n">
@@ -2414,10 +2426,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I36" s="1" t="n">
+      <c r="I36" s="2" t="n">
         <v>45975</v>
       </c>
-      <c r="J36" s="1" t="n">
+      <c r="J36" s="2" t="n">
         <v>45979</v>
       </c>
       <c r="K36" t="n">
@@ -2471,10 +2483,10 @@
           <t>Emma</t>
         </is>
       </c>
-      <c r="I37" s="1" t="n">
+      <c r="I37" s="2" t="n">
         <v>45978</v>
       </c>
-      <c r="J37" s="1" t="n">
+      <c r="J37" s="2" t="n">
         <v>45994</v>
       </c>
       <c r="K37" t="n">
@@ -2528,10 +2540,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I38" s="1" t="n">
+      <c r="I38" s="2" t="n">
         <v>45979</v>
       </c>
-      <c r="J38" s="1" t="n">
+      <c r="J38" s="2" t="n">
         <v>45981</v>
       </c>
       <c r="K38" t="n">
@@ -2585,10 +2597,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I39" s="1" t="n">
+      <c r="I39" s="2" t="n">
         <v>45981</v>
       </c>
-      <c r="J39" s="1" t="n">
+      <c r="J39" s="2" t="n">
         <v>46034</v>
       </c>
       <c r="K39" t="n">
@@ -2642,10 +2654,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I40" s="1" t="n">
+      <c r="I40" s="2" t="n">
         <v>45994</v>
       </c>
-      <c r="J40" s="1" t="n">
+      <c r="J40" s="2" t="n">
         <v>45999</v>
       </c>
       <c r="K40" t="n">
@@ -2699,10 +2711,10 @@
           <t>Emma</t>
         </is>
       </c>
-      <c r="I41" s="1" t="n">
+      <c r="I41" s="2" t="n">
         <v>45994</v>
       </c>
-      <c r="J41" s="1" t="n">
+      <c r="J41" s="2" t="n">
         <v>46001</v>
       </c>
       <c r="K41" t="n">
@@ -2756,10 +2768,10 @@
           <t>Shannon</t>
         </is>
       </c>
-      <c r="I42" s="1" t="n">
+      <c r="I42" s="2" t="n">
         <v>45994</v>
       </c>
-      <c r="J42" s="1" t="n">
+      <c r="J42" s="2" t="n">
         <v>46001</v>
       </c>
       <c r="K42" t="n">
@@ -2813,10 +2825,10 @@
           <t>Shannon</t>
         </is>
       </c>
-      <c r="I43" s="1" t="n">
+      <c r="I43" s="2" t="n">
         <v>46001</v>
       </c>
-      <c r="J43" s="1" t="n">
+      <c r="J43" s="2" t="n">
         <v>46006</v>
       </c>
       <c r="K43" t="n">
@@ -2870,10 +2882,10 @@
           <t>Emma</t>
         </is>
       </c>
-      <c r="I44" s="1" t="n">
+      <c r="I44" s="2" t="n">
         <v>46001</v>
       </c>
-      <c r="J44" s="1" t="n">
+      <c r="J44" s="2" t="n">
         <v>46014</v>
       </c>
       <c r="K44" t="n">
@@ -2927,10 +2939,10 @@
           <t>Shannon</t>
         </is>
       </c>
-      <c r="I45" s="1" t="n">
+      <c r="I45" s="2" t="n">
         <v>46006</v>
       </c>
-      <c r="J45" s="1" t="n">
+      <c r="J45" s="2" t="n">
         <v>46015</v>
       </c>
       <c r="K45" t="n">
@@ -2984,10 +2996,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I46" s="1" t="n">
+      <c r="I46" s="2" t="n">
         <v>46010</v>
       </c>
-      <c r="J46" s="1" t="n">
+      <c r="J46" s="2" t="n">
         <v>46021</v>
       </c>
       <c r="K46" t="n">
@@ -3041,10 +3053,10 @@
           <t>Emma</t>
         </is>
       </c>
-      <c r="I47" s="1" t="n">
+      <c r="I47" s="2" t="n">
         <v>46014</v>
       </c>
-      <c r="J47" s="1" t="n">
+      <c r="J47" s="2" t="n">
         <v>46020</v>
       </c>
       <c r="K47" t="n">
@@ -3098,10 +3110,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I48" s="1" t="n">
+      <c r="I48" s="2" t="n">
         <v>46024</v>
       </c>
-      <c r="J48" s="1" t="n">
+      <c r="J48" s="2" t="n">
         <v>46027</v>
       </c>
       <c r="K48" t="n">
@@ -3155,10 +3167,10 @@
           <t>Emma</t>
         </is>
       </c>
-      <c r="I49" s="1" t="n">
+      <c r="I49" s="2" t="n">
         <v>46027</v>
       </c>
-      <c r="J49" s="1" t="n">
+      <c r="J49" s="2" t="n">
         <v>46036</v>
       </c>
       <c r="K49" t="n">
@@ -3212,10 +3224,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I50" s="1" t="n">
+      <c r="I50" s="2" t="n">
         <v>46028</v>
       </c>
-      <c r="J50" s="1" t="n">
+      <c r="J50" s="2" t="n">
         <v>46034</v>
       </c>
       <c r="K50" t="n">
@@ -3269,10 +3281,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I51" s="1" t="n">
+      <c r="I51" s="2" t="n">
         <v>46035</v>
       </c>
-      <c r="J51" s="1" t="n">
+      <c r="J51" s="2" t="n">
         <v>46038</v>
       </c>
       <c r="K51" t="n">
@@ -3326,10 +3338,10 @@
           <t>Emma</t>
         </is>
       </c>
-      <c r="I52" s="1" t="n">
+      <c r="I52" s="2" t="n">
         <v>46038</v>
       </c>
-      <c r="J52" s="1" t="n">
+      <c r="J52" s="2" t="n">
         <v>46045</v>
       </c>
       <c r="K52" t="n">
@@ -3349,7 +3361,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Amenity Hub Tampa Phase 2</t>
+          <t>Amenity ADP Hub Tampa Phase 2</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3364,7 +3376,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Amenity</t>
+          <t>Amenity ADP</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -3383,10 +3395,10 @@
           <t>Shannon</t>
         </is>
       </c>
-      <c r="I53" s="1" t="n">
+      <c r="I53" s="2" t="n">
         <v>46042</v>
       </c>
-      <c r="J53" s="1" t="n">
+      <c r="J53" s="2" t="n">
         <v>46048</v>
       </c>
       <c r="K53" t="n">
@@ -3440,10 +3452,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I54" s="1" t="n">
+      <c r="I54" s="2" t="n">
         <v>46043</v>
       </c>
-      <c r="J54" s="1" t="n">
+      <c r="J54" s="2" t="n">
         <v>46048</v>
       </c>
       <c r="K54" t="n">
@@ -3493,10 +3505,10 @@
           <t>Emma</t>
         </is>
       </c>
-      <c r="I55" s="1" t="n">
+      <c r="I55" s="2" t="n">
         <v>46045</v>
       </c>
-      <c r="J55" s="1" t="n">
+      <c r="J55" s="2" t="n">
         <v>46046</v>
       </c>
       <c r="K55" t="n">
@@ -3550,10 +3562,10 @@
           <t>Shannon</t>
         </is>
       </c>
-      <c r="I56" s="1" t="n">
+      <c r="I56" s="2" t="n">
         <v>46048</v>
       </c>
-      <c r="J56" s="1" t="n">
+      <c r="J56" s="2" t="n">
         <v>46051</v>
       </c>
       <c r="K56" t="n">
@@ -3607,10 +3619,10 @@
           <t>Emma</t>
         </is>
       </c>
-      <c r="I57" s="1" t="n">
+      <c r="I57" s="2" t="n">
         <v>46049</v>
       </c>
-      <c r="J57" s="1" t="n">
+      <c r="J57" s="2" t="n">
         <v>46051</v>
       </c>
       <c r="K57" t="n">
@@ -3664,10 +3676,10 @@
           <t>Emma</t>
         </is>
       </c>
-      <c r="I58" s="1" t="n">
+      <c r="I58" s="2" t="n">
         <v>46052</v>
       </c>
-      <c r="J58" s="1" t="n">
+      <c r="J58" s="2" t="n">
         <v>46066</v>
       </c>
       <c r="K58" t="n">
@@ -3717,10 +3729,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I59" s="1" t="n">
+      <c r="I59" s="2" t="n">
         <v>46058</v>
       </c>
-      <c r="J59" s="1" t="n">
+      <c r="J59" s="2" t="n">
         <v>46066</v>
       </c>
       <c r="K59" t="n">
@@ -3770,10 +3782,10 @@
           <t>Shannon</t>
         </is>
       </c>
-      <c r="I60" s="1" t="n">
+      <c r="I60" s="2" t="n">
         <v>46063</v>
       </c>
-      <c r="J60" s="1" t="n">
+      <c r="J60" s="2" t="n">
         <v>46069</v>
       </c>
       <c r="K60" t="n">
@@ -3827,10 +3839,10 @@
           <t>Emma</t>
         </is>
       </c>
-      <c r="I61" s="1" t="n">
+      <c r="I61" s="2" t="n">
         <v>46063</v>
       </c>
-      <c r="J61" s="1" t="n">
+      <c r="J61" s="2" t="n">
         <v>46070</v>
       </c>
       <c r="K61" t="n">
@@ -3884,10 +3896,10 @@
           <t>Shannon</t>
         </is>
       </c>
-      <c r="I62" s="1" t="n">
+      <c r="I62" s="2" t="n">
         <v>46069</v>
       </c>
-      <c r="J62" s="1" t="n">
+      <c r="J62" s="2" t="n">
         <v>46072</v>
       </c>
       <c r="K62" t="n">
@@ -3937,10 +3949,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I63" s="1" t="n">
+      <c r="I63" s="2" t="n">
         <v>46069</v>
       </c>
-      <c r="J63" s="1" t="n">
+      <c r="J63" s="2" t="n">
         <v>46077</v>
       </c>
       <c r="K63" t="n">
@@ -3994,10 +4006,10 @@
           <t>Shannon</t>
         </is>
       </c>
-      <c r="I64" s="1" t="n">
+      <c r="I64" s="2" t="n">
         <v>46069</v>
       </c>
-      <c r="J64" s="1" t="n">
+      <c r="J64" s="2" t="n">
         <v>46083</v>
       </c>
       <c r="K64" t="n">
@@ -4051,10 +4063,10 @@
           <t>Shannon</t>
         </is>
       </c>
-      <c r="I65" s="1" t="n">
+      <c r="I65" s="2" t="n">
         <v>46069</v>
       </c>
-      <c r="J65" s="1" t="n">
+      <c r="J65" s="2" t="n">
         <v>46083</v>
       </c>
       <c r="K65" t="n">
@@ -4108,10 +4120,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I66" s="1" t="n">
+      <c r="I66" s="2" t="n">
         <v>46076</v>
       </c>
-      <c r="J66" s="1" t="n">
+      <c r="J66" s="2" t="n">
         <v>46078</v>
       </c>
       <c r="K66" t="n">
@@ -4165,10 +4177,10 @@
           <t>Neil</t>
         </is>
       </c>
-      <c r="I67" s="1" t="n">
+      <c r="I67" s="2" t="n">
         <v>46076</v>
       </c>
-      <c r="J67" s="1" t="n">
+      <c r="J67" s="2" t="n">
         <v>46078</v>
       </c>
       <c r="K67" t="n">
@@ -4188,45 +4200,49 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>MAIN #3 320 Lakeview Ave</t>
+          <t>SWBD Main 1 St Regis Residences Brickell (fka 1809 Brickell Ave)</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>320 Lakeview Ave</t>
+          <t>St Regis Residences Brickell (fka 1809 Brickell Ave)</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>SM25-203</t>
+          <t>SM25-245</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>MAIN #3</t>
+          <t>SWBD Main 1</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>277/480v 3PH 4W 3000a BUS 3000a ARMS LSIG MCB 65 KAIC</t>
+          <t xml:space="preserve">120/208V 3PH 4W 4000a MCB 100 KAIC NEMA 1 </t>
         </is>
       </c>
       <c r="F68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G68" t="n">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Neil</t>
-        </is>
-      </c>
-      <c r="I68" s="1" t="n">
-        <v>46079</v>
-      </c>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
+          <t>Shannon</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="n">
+        <v>46084</v>
+      </c>
+      <c r="J68" s="2" t="n">
+        <v>46097</v>
+      </c>
+      <c r="K68" t="n">
+        <v>13</v>
+      </c>
       <c r="L68" t="inlineStr">
         <is>
           <t>Easy</t>
@@ -4241,48 +4257,48 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SWBD Main 1 St Regis Residences Brickell (fka 1809 Brickell Ave)</t>
+          <t>NMSBH Ritz Carlton Res Bay P2</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>St Regis Residences Brickell (fka 1809 Brickell Ave)</t>
+          <t>Ritz Carlton Res Bay P2</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>SM25-245</t>
+          <t>SM25-210</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>SWBD Main 1</t>
+          <t>NMSBH</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t xml:space="preserve">120/208V 3PH 4W 4000a MCB 100 KAIC NEMA 1 </t>
+          <t xml:space="preserve">277/480v 3PH 4W 3000a BUS 3000a ARMS MCB 65 KAIC NEMA 1 </t>
         </is>
       </c>
       <c r="F69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G69" t="n">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Shannon</t>
-        </is>
-      </c>
-      <c r="I69" s="1" t="n">
-        <v>46084</v>
-      </c>
-      <c r="J69" s="1" t="n">
+          <t>Neil</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="n">
+        <v>46091</v>
+      </c>
+      <c r="J69" s="2" t="n">
         <v>46097</v>
       </c>
       <c r="K69" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="L69" t="inlineStr">
         <is>
@@ -4298,52 +4314,52 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>NMSBH Ritz Carlton Res Bay P2</t>
+          <t>HDP Main 4 St Regis Residences Brickell (fka 1809 Brickell Ave)</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Ritz Carlton Res Bay P2</t>
+          <t>St Regis Residences Brickell (fka 1809 Brickell Ave)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>SM25-210</t>
+          <t>SM25-133</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>NMSBH</t>
+          <t>HDP Main 4</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t xml:space="preserve">277/480v 3PH 4W 3000a BUS 3000a ARMS MCB 65 KAIC NEMA 1 </t>
+          <t>480/277V 3PH 4W 4000a MCB 100 KAIC NEMA 1</t>
         </is>
       </c>
       <c r="F70" t="n">
         <v>3</v>
       </c>
       <c r="G70" t="n">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Neil</t>
-        </is>
-      </c>
-      <c r="I70" s="1" t="n">
-        <v>46091</v>
-      </c>
-      <c r="J70" s="1" t="n">
+          <t>Shannon</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="n">
         <v>46097</v>
       </c>
+      <c r="J70" s="2" t="n">
+        <v>46098</v>
+      </c>
       <c r="K70" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>Easy</t>
+          <t>Med</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
@@ -4355,52 +4371,52 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>HDP Main 4 St Regis Residences Brickell (fka 1809 Brickell Ave)</t>
+          <t>EQMH Bentley Residences</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>St Regis Residences Brickell (fka 1809 Brickell Ave)</t>
+          <t>Bentley Residences</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>SM25-133</t>
+          <t>SM25-191</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>HDP Main 4</t>
+          <t>EQMH</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>480/277V 3PH 4W 4000a MCB 100 KAIC NEMA 1</t>
+          <t xml:space="preserve">480/277v 3ph 4w 1600a MLO 65KAIC NEMA 3R </t>
         </is>
       </c>
       <c r="F71" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G71" t="n">
-        <v>4000</v>
+        <v>1600</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Shannon</t>
-        </is>
-      </c>
-      <c r="I71" s="1" t="n">
+          <t>Micah</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="n">
         <v>46097</v>
       </c>
-      <c r="J71" s="1" t="n">
-        <v>46098</v>
+      <c r="J71" s="2" t="n">
+        <v>46101</v>
       </c>
       <c r="K71" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
@@ -4412,48 +4428,48 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>EQMH Bentley Residences</t>
+          <t>NMSBE Ritz Carlton Res Bay P2</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Bentley Residences</t>
+          <t>Ritz Carlton Res Bay P2</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>SM25-191</t>
+          <t>SM25-210</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>EQMH</t>
+          <t>NMSBE</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t xml:space="preserve">480/277v 3ph 4w 1600a MLO 65KAIC NEMA 3R </t>
+          <t xml:space="preserve">277/480v 3PH 4W 1600a BUS 1600a GFP MCB 65 KAIC NEMA 1 </t>
         </is>
       </c>
       <c r="F72" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G72" t="n">
         <v>1600</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Micah</t>
-        </is>
-      </c>
-      <c r="I72" s="1" t="n">
-        <v>46097</v>
-      </c>
-      <c r="J72" s="1" t="n">
-        <v>46101</v>
+          <t>Neil</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="n">
+        <v>46098</v>
+      </c>
+      <c r="J72" s="2" t="n">
+        <v>46104</v>
       </c>
       <c r="K72" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L72" t="inlineStr">
         <is>
@@ -4469,45 +4485,45 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>NMSBE Ritz Carlton Res Bay P2</t>
+          <t>Car Charge Main 1 St Regis Residences Brickell (fka 1809 Brickell Ave)</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Ritz Carlton Res Bay P2</t>
+          <t>St Regis Residences Brickell (fka 1809 Brickell Ave)</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>SM25-210</t>
+          <t>SM25-133</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>NMSBE</t>
+          <t>Car Charge Main 1</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t xml:space="preserve">277/480v 3PH 4W 1600a BUS 1600a GFP MCB 65 KAIC NEMA 1 </t>
+          <t xml:space="preserve">120/208V 3PH 4W 2000a MCB 100 KAIC NEMA 1 </t>
         </is>
       </c>
       <c r="F73" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G73" t="n">
-        <v>1600</v>
+        <v>2000</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Neil</t>
-        </is>
-      </c>
-      <c r="I73" s="1" t="n">
-        <v>46098</v>
-      </c>
-      <c r="J73" s="1" t="n">
-        <v>46104</v>
+          <t>Shannon</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="n">
+        <v>46099</v>
+      </c>
+      <c r="J73" s="2" t="n">
+        <v>46105</v>
       </c>
       <c r="K73" t="n">
         <v>6</v>
@@ -4526,27 +4542,27 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Car Charge Main 1 St Regis Residences Brickell (fka 1809 Brickell Ave)</t>
+          <t>EMOP Bentley Residences</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>St Regis Residences Brickell (fka 1809 Brickell Ave)</t>
+          <t>Bentley Residences</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>SM25-133</t>
+          <t>SM25-131.01</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Car Charge Main 1</t>
+          <t>EMOP</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t xml:space="preserve">120/208V 3PH 4W 2000a MCB 100 KAIC NEMA 1 </t>
+          <t>120/208v 3PH 4W 2000a MLO 65 KAIC NEMA 1</t>
         </is>
       </c>
       <c r="F74" t="n">
@@ -4557,17 +4573,17 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Shannon</t>
-        </is>
-      </c>
-      <c r="I74" s="1" t="n">
-        <v>46099</v>
-      </c>
-      <c r="J74" s="1" t="n">
-        <v>46105</v>
+          <t>Micah</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="n">
+        <v>46101</v>
+      </c>
+      <c r="J74" s="2" t="n">
+        <v>46104</v>
       </c>
       <c r="K74" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L74" t="inlineStr">
         <is>
@@ -4583,48 +4599,48 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>EMOP Bentley Residences</t>
+          <t>NMSBR Ritz Carlton Res Bay P2</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Bentley Residences</t>
+          <t>Ritz Carlton Res Bay P2</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>SM25-131.01</t>
+          <t>SM25-210</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>EMOP</t>
+          <t>NMSBR</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>120/208v 3PH 4W 2000a MLO 65 KAIC NEMA 1</t>
+          <t xml:space="preserve">120/208v 3PH 4W 4000a BUS 4000a ARMS MLO 65 KAIC NEMA 1 </t>
         </is>
       </c>
       <c r="F75" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G75" t="n">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Micah</t>
-        </is>
-      </c>
-      <c r="I75" s="1" t="n">
-        <v>46101</v>
-      </c>
-      <c r="J75" s="1" t="n">
+          <t>Neil</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="n">
         <v>46104</v>
       </c>
+      <c r="J75" s="2" t="n">
+        <v>46120</v>
+      </c>
       <c r="K75" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -4640,48 +4656,48 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>NMSBR Ritz Carlton Res Bay P2</t>
+          <t>EMSB Bentley Residences</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Ritz Carlton Res Bay P2</t>
+          <t>Bentley Residences</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>SM25-210</t>
+          <t>SM25-274</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>NMSBR</t>
+          <t>EMSB</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t xml:space="preserve">120/208v 3PH 4W 4000a BUS 4000a ARMS MLO 65 KAIC NEMA 1 </t>
+          <t xml:space="preserve">480/277v 3PH 4W 4000a BUS 4000a ERMS MCB 65 KAIC NEMA 1 </t>
         </is>
       </c>
       <c r="F76" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G76" t="n">
         <v>4000</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Neil</t>
-        </is>
-      </c>
-      <c r="I76" s="1" t="n">
-        <v>46104</v>
-      </c>
-      <c r="J76" s="1" t="n">
-        <v>46120</v>
+          <t>Micah</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="n">
+        <v>46105</v>
+      </c>
+      <c r="J76" s="2" t="n">
+        <v>46118</v>
       </c>
       <c r="K76" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="L76" t="inlineStr">
         <is>
@@ -4731,10 +4747,10 @@
           <t>Shannon</t>
         </is>
       </c>
-      <c r="I77" s="1" t="n">
+      <c r="I77" s="2" t="n">
         <v>46108</v>
       </c>
-      <c r="J77" s="1" t="n">
+      <c r="J77" s="2" t="n">
         <v>46118</v>
       </c>
       <c r="K77" t="n">
@@ -4788,10 +4804,10 @@
           <t>Shannon</t>
         </is>
       </c>
-      <c r="I78" s="1" t="n">
+      <c r="I78" s="2" t="n">
         <v>46108</v>
       </c>
-      <c r="J78" s="1" t="n">
+      <c r="J78" s="2" t="n">
         <v>46118</v>
       </c>
       <c r="K78" t="n">
@@ -4845,10 +4861,10 @@
           <t>Shannon</t>
         </is>
       </c>
-      <c r="I79" s="1" t="n">
+      <c r="I79" s="2" t="n">
         <v>46108</v>
       </c>
-      <c r="J79" s="1" t="n">
+      <c r="J79" s="2" t="n">
         <v>46118</v>
       </c>
       <c r="K79" t="n">
@@ -4902,10 +4918,10 @@
           <t>Shannon</t>
         </is>
       </c>
-      <c r="I80" s="1" t="n">
+      <c r="I80" s="2" t="n">
         <v>46108</v>
       </c>
-      <c r="J80" s="1" t="n">
+      <c r="J80" s="2" t="n">
         <v>46118</v>
       </c>
       <c r="K80" t="n">
@@ -4959,10 +4975,10 @@
           <t>Shannon</t>
         </is>
       </c>
-      <c r="I81" s="1" t="n">
+      <c r="I81" s="2" t="n">
         <v>46118</v>
       </c>
-      <c r="J81" s="1" t="n">
+      <c r="J81" s="2" t="n">
         <v>46125</v>
       </c>
       <c r="K81" t="n">
@@ -4976,6 +4992,458 @@
       <c r="M81" t="inlineStr">
         <is>
           <t>2026Q2</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>ROSH Bentley Residences</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Bentley Residences</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>SM25-191</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>ROSH</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">120/208v 3PH 4W 2500a BUS  MLO 65 KAIC NEMA 1 </t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>2</v>
+      </c>
+      <c r="G82" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Shannon</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="n">
+        <v>46125</v>
+      </c>
+      <c r="J82" s="2" t="n">
+        <v>46134</v>
+      </c>
+      <c r="K82" t="n">
+        <v>9</v>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>2026Q2</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>DPH-07F  Santander Tower (aka 1401 Brickell)</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Santander Tower (aka 1401 Brickell)</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>SM25-232</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DPH-07F </t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>277/480v 3PH 4W 2000a BUS 2000a ARMS MCB 65 KAIC NEMA 1</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>2</v>
+      </c>
+      <c r="G83" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Steven</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="n">
+        <v>46127</v>
+      </c>
+      <c r="J83" s="2" t="n">
+        <v>46128</v>
+      </c>
+      <c r="K83" t="n">
+        <v>1</v>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>2026Q2</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>RDPH Bentley Residences</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Bentley Residences</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>SM25-191</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>RDPH</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">480/277v 3PH 4W 2500a MLO 65 KAIC NEMA 1 </t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>2</v>
+      </c>
+      <c r="G84" t="n">
+        <v>2500</v>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Shannon</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="n">
+        <v>46127</v>
+      </c>
+      <c r="J84" s="2" t="n">
+        <v>46132</v>
+      </c>
+      <c r="K84" t="n">
+        <v>5</v>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>2026Q2</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>DPH-RA  Santander Tower (aka 1401 Brickell)</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Santander Tower (aka 1401 Brickell)</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>SM25-232</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DPH-RA </t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">277/480v 3PH 4W 2000a BUS 2000a GFP MCB 65 KAIC NEMA 1 </t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>2</v>
+      </c>
+      <c r="G85" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Steven</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="n">
+        <v>46129</v>
+      </c>
+      <c r="J85" s="2" t="n">
+        <v>46132</v>
+      </c>
+      <c r="K85" t="n">
+        <v>3</v>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>2026Q2</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>E2DPH-07A  Santander Tower (aka 1401 Brickell)</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Santander Tower (aka 1401 Brickell)</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>SM25-232</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E2DPH-07A </t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">277/480v 3PH 4W 2000a BUS 2000a ARMS MCB 65 KAIC NEMA 1 </t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>2</v>
+      </c>
+      <c r="G86" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Steven</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="n">
+        <v>46133</v>
+      </c>
+      <c r="J86" s="2" t="n">
+        <v>46134</v>
+      </c>
+      <c r="K86" t="n">
+        <v>1</v>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>2026Q2</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>GSB-1  The Reserve at Strathmore Square</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>The Reserve at Strathmore Square</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>SM25-275</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GSB-1 </t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>277/480v 3PH 4W 1600a BUS 1600a MLO 65 KAIC</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>3</v>
+      </c>
+      <c r="G87" t="n">
+        <v>1600</v>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Steven</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="n">
+        <v>46133</v>
+      </c>
+      <c r="J87" s="2" t="n">
+        <v>46134</v>
+      </c>
+      <c r="K87" t="n">
+        <v>1</v>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>2026Q2</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>TGDP  The Reserve at Strathmore Square</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>The Reserve at Strathmore Square</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>SM25-275</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TGDP </t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>277/480v 3PH 4W 1200a BUS 1200a MLO 65 KAIC</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>2</v>
+      </c>
+      <c r="G88" t="n">
+        <v>1200</v>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Steven</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="n">
+        <v>46133</v>
+      </c>
+      <c r="J88" s="2" t="n">
+        <v>46134</v>
+      </c>
+      <c r="K88" t="n">
+        <v>1</v>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>2026Q2</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>GDP 8th St. Brickell (Sentral Brickell)</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>8th St. Brickell (Sentral Brickell)</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>SM25-131</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>GDP</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">480/277V 3PH 4W 2000a MCB 100 KAIC NEMA 1 </t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>1</v>
+      </c>
+      <c r="G89" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Steven</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" s="2" t="n">
+        <v>46125</v>
+      </c>
+      <c r="K89" t="inlineStr"/>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>NaT</t>
         </is>
       </c>
     </row>

</xml_diff>